<commit_message>
Ajout du calcul du chauffage dans l'explication des charges
</commit_message>
<xml_diff>
--- a/data/Modele.xlsx
+++ b/data/Modele.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="270" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{681B539C-AB20-4DB7-84CF-ABF379C2454E}"/>
+  <xr:revisionPtr revIDLastSave="275" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86858F62-3398-47FE-94B0-E244F94D5BA8}"/>
   <bookViews>
-    <workbookView xWindow="3870" yWindow="4935" windowWidth="28800" windowHeight="15345" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenus" sheetId="3" r:id="rId1"/>
@@ -734,10 +734,10 @@
     <t>Lot 308 - T2 2ème étage Batiment 3 exposé ouest</t>
   </si>
   <si>
+    <t>Lot 113</t>
+  </si>
+  <si>
     <t>Lot 134</t>
-  </si>
-  <si>
-    <t>Lot 113</t>
   </si>
 </sst>
 </file>
@@ -810,87 +810,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Monétaire" xfId="1" builtinId="4"/>
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Pourcentage" xfId="2" builtinId="5"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="26">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1178,6 +1102,82 @@
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1196,7 +1196,7 @@
   <autoFilter ref="A1:B2" xr:uid="{B8BAE385-571F-4715-A042-0AD7A1FDF085}"/>
   <tableColumns count="2">
     <tableColumn id="2" xr3:uid="{75AB35E7-AA7F-46C7-B30C-DC2E9C862FFF}" name="Label du revenu"/>
-    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1213,7 +1213,7 @@
     <tableColumn id="5" xr3:uid="{F17C785C-9055-484D-A7EC-C3372D32A622}" name="Segment"/>
     <tableColumn id="7" xr3:uid="{3DB4DC80-D06E-4E70-BFE9-9BB75CB5FA62}" name="Classe de provision"/>
     <tableColumn id="2" xr3:uid="{3B6645ED-EDB5-4F76-9846-790ECF4F680D}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="25" totalsRowDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1226,16 +1226,16 @@
     <sortCondition ref="B1:B47"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="20"/>
     <tableColumn id="3" xr3:uid="{5B85ADF0-B113-45E5-864A-388F8040031F}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="2">
+    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="17">
       <calculatedColumnFormula>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1248,23 +1248,23 @@
     <tableColumn id="12" xr3:uid="{6157D014-929F-42D7-A4BC-12D951282608}" name="Batiment"/>
     <tableColumn id="4" xr3:uid="{81B9BF77-9818-477B-B3E8-1E987064DFDA}" name="Label de lot"/>
     <tableColumn id="1" xr3:uid="{B1F46291-565B-462F-9110-123FFF38DDEE}" name="Nom du coproprietaire"/>
-    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="25">
+    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="15">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="24"/>
-    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="23"/>
-    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="22"/>
-    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="21"/>
-    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="20"/>
-    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="19"/>
-    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="18"/>
-    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="17"/>
-    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="16"/>
-    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="15"/>
-    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="14"/>
-    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="11"/>
+    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="10"/>
+    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="9"/>
+    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="8"/>
+    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="7"/>
+    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="6"/>
+    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="4"/>
+    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{71861424-FDE4-4C97-8393-5794B9911F90}" name="Lot Nexity"/>
     <tableColumn id="5" xr3:uid="{99825B0E-48FC-48C3-B40C-A8763FC406C7}" name="Etage"/>
   </tableColumns>
@@ -1551,13 +1551,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9248CCDF-C1D7-473F-904E-6A9FA3872F9C}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="33.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="33.7265625" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>122</v>
       </c>
@@ -1565,7 +1565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1587,16 +1587,16 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:E35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.81640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>110</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>103</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>104</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>190</v>
       </c>
@@ -1658,13 +1658,13 @@
         <v>197</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>197</v>
       </c>
       <c r="E4" s="1">
         <v>2000</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>105</v>
       </c>
@@ -1681,7 +1681,7 @@
         <v>2900</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>191</v>
       </c>
@@ -1692,13 +1692,13 @@
         <v>198</v>
       </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>198</v>
       </c>
       <c r="E6" s="1">
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>106</v>
       </c>
@@ -1715,7 +1715,7 @@
         <v>2900</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>192</v>
       </c>
@@ -1726,13 +1726,13 @@
         <v>199</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>199</v>
       </c>
       <c r="E8" s="1">
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>84</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>83</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>6200</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>80</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>79</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>78</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>71</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>72</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>81</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>86</v>
       </c>
@@ -1885,7 +1885,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>87</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>76</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>75</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>73</v>
       </c>
@@ -1953,7 +1953,7 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -1985,7 +1985,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>82</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>85</v>
       </c>
@@ -2019,7 +2019,7 @@
         <v>16800</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>95</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>89</v>
       </c>
@@ -2053,7 +2053,7 @@
         <v>23100</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>88</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>90</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>17650</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>92</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>91</v>
       </c>
@@ -2121,7 +2121,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>93</v>
       </c>
@@ -2138,7 +2138,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>107</v>
       </c>
@@ -2155,7 +2155,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>94</v>
       </c>
@@ -2172,7 +2172,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="D35"/>
       <c r="E35" s="4">
         <f>SUBTOTAL(109,BdBudgetPrevisionnel[Provision])</f>
@@ -2193,19 +2193,19 @@
     <tabColor theme="7" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:I47"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="48.140625" customWidth="1"/>
-    <col min="2" max="2" width="66.5703125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="159.7109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="48.1796875" customWidth="1"/>
+    <col min="2" max="2" width="66.54296875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="32.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.26953125" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="159.7265625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>130</v>
       </c>
@@ -2231,7 +2231,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>28</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>209</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>208</v>
       </c>
@@ -2306,7 +2306,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>200</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>209</v>
       </c>
@@ -2360,7 +2360,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>208</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>200</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>209</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>208</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>200</v>
       </c>
@@ -2495,7 +2495,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>209</v>
       </c>
@@ -2522,7 +2522,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>208</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>10</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>10</v>
       </c>
@@ -2699,7 +2699,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>25</v>
       </c>
@@ -2727,7 +2727,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>25</v>
       </c>
@@ -2755,7 +2755,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>25</v>
       </c>
@@ -2779,7 +2779,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>25</v>
       </c>
@@ -2803,7 +2803,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>17</v>
       </c>
@@ -2831,7 +2831,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>17</v>
       </c>
@@ -2859,7 +2859,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>17</v>
       </c>
@@ -2887,7 +2887,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>23</v>
       </c>
@@ -2914,7 +2914,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>23</v>
       </c>
@@ -2941,7 +2941,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>23</v>
       </c>
@@ -2968,7 +2968,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>18</v>
       </c>
@@ -2995,7 +2995,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>18</v>
       </c>
@@ -3022,7 +3022,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>18</v>
       </c>
@@ -3049,7 +3049,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>18</v>
       </c>
@@ -3076,7 +3076,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>30</v>
       </c>
@@ -3097,7 +3097,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>17</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>17</v>
       </c>
@@ -3153,7 +3153,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>19</v>
       </c>
@@ -3174,7 +3174,7 @@
         <v>3198.13</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>19</v>
       </c>
@@ -3195,7 +3195,7 @@
         <v>3322.8</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>19</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>3138.27</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>18</v>
       </c>
@@ -3243,7 +3243,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>18</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>18</v>
       </c>
@@ -3297,7 +3297,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>18</v>
       </c>
@@ -3324,7 +3324,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>124</v>
       </c>
@@ -3350,7 +3350,7 @@
       <c r="H44" s="5"/>
       <c r="I44" s="2"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>124</v>
       </c>
@@ -3376,7 +3376,7 @@
       <c r="H45" s="5"/>
       <c r="I45" s="2"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>124</v>
       </c>
@@ -3402,7 +3402,7 @@
       <c r="H46" s="5"/>
       <c r="I46" s="2"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>124</v>
       </c>
@@ -3456,25 +3456,25 @@
     <tabColor theme="2" tint="-9.9978637043366805E-2"/>
   </sheetPr>
   <dimension ref="A1:T7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="48.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="12" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="25.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="12" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="37.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>174</v>
       </c>
@@ -3536,7 +3536,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>59</v>
       </c>
@@ -3579,7 +3579,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -3620,7 +3620,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>57</v>
       </c>
@@ -3628,7 +3628,7 @@
         <v>173</v>
       </c>
       <c r="C4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D4" s="10">
         <v>102</v>
@@ -3666,7 +3666,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -3674,7 +3674,7 @@
         <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D5" s="10">
         <v>7</v>
@@ -3708,7 +3708,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -3716,7 +3716,7 @@
         <v>173</v>
       </c>
       <c r="C6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D6" s="10">
         <v>86</v>
@@ -3754,7 +3754,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>70</v>
       </c>
@@ -3762,7 +3762,7 @@
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D7" s="10">
         <v>7</v>
@@ -3811,14 +3811,14 @@
     <tabColor theme="2" tint="-9.9978637043366805E-2"/>
   </sheetPr>
   <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="90.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="90.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>117</v>
       </c>
@@ -3832,7 +3832,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -3847,7 +3847,7 @@
         <v>-600</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3862,7 +3862,7 @@
         <v>-1800</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3877,7 +3877,7 @@
         <v>-5000</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -3886,7 +3886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>36</v>
       </c>
@@ -3895,7 +3895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -3913,7 +3913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>39</v>
       </c>

</xml_diff>

<commit_message>
On enlève les feuilles inutiles du fichier Excel
</commit_message>
<xml_diff>
--- a/data/Modele.xlsx
+++ b/data/Modele.xlsx
@@ -8,16 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="275" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86858F62-3398-47FE-94B0-E244F94D5BA8}"/>
+  <xr:revisionPtr revIDLastSave="277" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7EF880B-72ED-40D8-AE0D-7B40117B1E3F}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Revenus" sheetId="3" r:id="rId1"/>
-    <sheet name="Budget" sheetId="7" r:id="rId2"/>
-    <sheet name="Propositions" sheetId="6" r:id="rId3"/>
-    <sheet name="Copropriétaires" sheetId="5" r:id="rId4"/>
-    <sheet name="Règles" sheetId="4" r:id="rId5"/>
+    <sheet name="Budget" sheetId="7" r:id="rId1"/>
+    <sheet name="Propositions" sheetId="6" r:id="rId2"/>
+    <sheet name="Copropriétaires" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,19 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="232">
-  <si>
-    <t>Montant</t>
-  </si>
-  <si>
-    <t>Avance de trésorerie</t>
-  </si>
-  <si>
-    <t>Montant d'un marché à partir duquel la consultation du conseil syndical est obligatoire</t>
-  </si>
-  <si>
-    <t>Montant d'un marché à partir duquel la mise en compétition est obligatoire</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="219">
   <si>
     <t>Taxes</t>
   </si>
@@ -66,9 +52,6 @@
     <t>Total TTC</t>
   </si>
   <si>
-    <t>Le conseil syndical peut dépenser cette somme au plus sans consulter les copropriétaires</t>
-  </si>
-  <si>
     <t>Cout</t>
   </si>
   <si>
@@ -147,21 +130,6 @@
     <t>ça coute combien ?</t>
   </si>
   <si>
-    <t>La police municipale peut pénétrer dans la résidence</t>
-  </si>
-  <si>
-    <t>Mandat de 4 ans au syndic pour renégocier le contrat de gaz auprès de KOPROWATT ENERGIES</t>
-  </si>
-  <si>
-    <t>Mandat de 4 ans au syndic pour renégocier le contrat d'électricité auprès de KOPROWATT ENERGIES</t>
-  </si>
-  <si>
-    <t>Accès en ligne aux infos de la copropriété</t>
-  </si>
-  <si>
-    <t>Réunion en vision Teams</t>
-  </si>
-  <si>
     <t>Eau froide</t>
   </si>
   <si>
@@ -393,12 +361,6 @@
     <t>Provision</t>
   </si>
   <si>
-    <t>Label des règles</t>
-  </si>
-  <si>
-    <t>Limite</t>
-  </si>
-  <si>
     <t>Label de lot</t>
   </si>
   <si>
@@ -406,9 +368,6 @@
   </si>
   <si>
     <t>Numéro de lot</t>
-  </si>
-  <si>
-    <t>Label du revenu</t>
   </si>
   <si>
     <t>Electricité de parties communes</t>
@@ -814,7 +773,47 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="24">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1102,82 +1101,6 @@
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1191,18 +1114,11 @@
 </styleSheet>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B8BAE385-571F-4715-A042-0AD7A1FDF085}" name="BdRevenus" displayName="BdRevenus" ref="A1:B2" totalsRowShown="0">
-  <autoFilter ref="A1:B2" xr:uid="{B8BAE385-571F-4715-A042-0AD7A1FDF085}"/>
-  <tableColumns count="2">
-    <tableColumn id="2" xr3:uid="{75AB35E7-AA7F-46C7-B30C-DC2E9C862FFF}" name="Label du revenu"/>
-    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="23"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{986F05D8-067A-4813-B8D0-1D3E83D9A8C6}" name="BdBudgetPrevisionnel" displayName="BdBudgetPrevisionnel" ref="A1:E35" totalsRowCount="1">
   <autoFilter ref="A1:E34" xr:uid="{986F05D8-067A-4813-B8D0-1D3E83D9A8C6}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E34">
@@ -1213,75 +1129,60 @@
     <tableColumn id="5" xr3:uid="{F17C785C-9055-484D-A7EC-C3372D32A622}" name="Segment"/>
     <tableColumn id="7" xr3:uid="{3DB4DC80-D06E-4E70-BFE9-9BB75CB5FA62}" name="Classe de provision"/>
     <tableColumn id="2" xr3:uid="{3B6645ED-EDB5-4F76-9846-790ECF4F680D}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="8" totalsRowDxfId="7"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1CA6001B-8A1B-4BBD-AB17-BC7D9D052A42}" name="BdCompetition" displayName="BdCompetition" ref="A1:H47" totalsRowShown="0">
+  <autoFilter ref="A1:H47" xr:uid="{1CA6001B-8A1B-4BBD-AB17-BC7D9D052A42}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H47">
+    <sortCondition ref="B1:B47"/>
+  </sortState>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{5B85ADF0-B113-45E5-864A-388F8040031F}" name="Prestataire"/>
+    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="1">
+      <calculatedColumnFormula>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1CA6001B-8A1B-4BBD-AB17-BC7D9D052A42}" name="BdCompetition" displayName="BdCompetition" ref="A1:H47" totalsRowShown="0">
-  <autoFilter ref="A1:H47" xr:uid="{1CA6001B-8A1B-4BBD-AB17-BC7D9D052A42}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H47">
-    <sortCondition ref="B1:B47"/>
-  </sortState>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{5B85ADF0-B113-45E5-864A-388F8040031F}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="17">
-      <calculatedColumnFormula>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="16"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3CEBCA3A-959D-43DA-A310-FB4D8334574B}" name="BdCoproprietaires" displayName="BdCoproprietaires" ref="A1:T7" totalsRowShown="0">
   <autoFilter ref="A1:T7" xr:uid="{3CEBCA3A-959D-43DA-A310-FB4D8334574B}"/>
   <tableColumns count="20">
     <tableColumn id="12" xr3:uid="{6157D014-929F-42D7-A4BC-12D951282608}" name="Batiment"/>
     <tableColumn id="4" xr3:uid="{81B9BF77-9818-477B-B3E8-1E987064DFDA}" name="Label de lot"/>
     <tableColumn id="1" xr3:uid="{B1F46291-565B-462F-9110-123FFF38DDEE}" name="Nom du coproprietaire"/>
-    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="15">
+    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="23">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="11"/>
-    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="10"/>
-    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="9"/>
-    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="8"/>
-    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="7"/>
-    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="6"/>
-    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="5"/>
-    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="4"/>
-    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="2"/>
-    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="19"/>
+    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="18"/>
+    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="17"/>
+    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="16"/>
+    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="15"/>
+    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="14"/>
+    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="13"/>
+    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="12"/>
+    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="10"/>
+    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="9"/>
     <tableColumn id="3" xr3:uid="{71861424-FDE4-4C97-8393-5794B9911F90}" name="Lot Nexity"/>
     <tableColumn id="5" xr3:uid="{99825B0E-48FC-48C3-B40C-A8763FC406C7}" name="Etage"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{594FE941-6967-448D-B161-1A22202460B2}" name="BdRegles" displayName="BdRegles" ref="A1:D9" totalsRowShown="0">
-  <autoFilter ref="A1:D9" xr:uid="{594FE941-6967-448D-B161-1A22202460B2}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{8584E7DE-3397-4839-B3F7-5BE29387C4A6}" name="Label des règles"/>
-    <tableColumn id="2" xr3:uid="{2DAB5E09-C6DA-4A52-9D36-12A8D2B9BE1E}" name="Limite" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{4C91DD63-5027-4E87-B95E-BCB801F28C1C}" name="Taxes"/>
-    <tableColumn id="4" xr3:uid="{41CB6CC9-60A9-4712-874D-13D61D2EB5DE}" name="Total TTC">
-      <calculatedColumnFormula>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</calculatedColumnFormula>
-    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1549,39 +1450,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9248CCDF-C1D7-473F-904E-6A9FA3872F9C}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="33.7265625" customWidth="1"/>
-    <col min="2" max="2" width="11.54296875" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>122</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1">
-        <v>25000</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B4565C1-1F2E-498D-BD21-D55E01D9459A}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
@@ -1598,33 +1466,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B1" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="C1" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="D1" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E2" s="1">
         <v>1500</v>
@@ -1632,16 +1500,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="D3" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="E3" s="1">
         <v>1500</v>
@@ -1649,16 +1517,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="D4" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="E4" s="1">
         <v>2000</v>
@@ -1666,16 +1534,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="D5" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="E5" s="1">
         <v>2900</v>
@@ -1683,16 +1551,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>198</v>
+        <v>185</v>
       </c>
       <c r="D6" t="s">
-        <v>198</v>
+        <v>185</v>
       </c>
       <c r="E6" s="1">
         <v>1000</v>
@@ -1700,16 +1568,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
-        <v>196</v>
+        <v>183</v>
       </c>
       <c r="D7" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="E7" s="1">
         <v>2900</v>
@@ -1717,16 +1585,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>192</v>
+        <v>179</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>199</v>
+        <v>186</v>
       </c>
       <c r="D8" t="s">
-        <v>199</v>
+        <v>186</v>
       </c>
       <c r="E8" s="1">
         <v>1000</v>
@@ -1734,16 +1602,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B9" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E9" s="1">
         <v>750</v>
@@ -1751,16 +1619,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E10" s="1">
         <v>6200</v>
@@ -1768,16 +1636,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="E11" s="1">
         <v>1050</v>
@@ -1785,16 +1653,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="B12" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C12" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E12" s="1">
         <v>900</v>
@@ -1802,16 +1670,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="B13" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D13" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E13" s="1">
         <v>920</v>
@@ -1819,16 +1687,16 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B14" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E14" s="1">
         <v>35000</v>
@@ -1836,16 +1704,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B15" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C15" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="D15" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="E15" s="1">
         <v>1500</v>
@@ -1853,16 +1721,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B16" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D16" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E16" s="1">
         <v>580</v>
@@ -1870,16 +1738,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="D17" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E17" s="1">
         <v>570</v>
@@ -1887,16 +1755,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C18" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="D18" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E18" s="1">
         <v>850</v>
@@ -1904,16 +1772,16 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="B19" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E19" s="1">
         <v>240</v>
@@ -1921,16 +1789,16 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C20" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="D20" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="E20" s="1">
         <v>220</v>
@@ -1938,16 +1806,16 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="B21" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="D21" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E21" s="1">
         <v>18000</v>
@@ -1955,31 +1823,31 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="B22" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C22" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D22" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E22" s="1"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C23" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D23" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="E23" s="1">
         <v>650</v>
@@ -1987,16 +1855,16 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="B24" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C24" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D24" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E24" s="1">
         <v>3500</v>
@@ -2004,16 +1872,16 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B25" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C25" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D25" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E25" s="1">
         <v>16800</v>
@@ -2021,16 +1889,16 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B26" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="C26" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D26" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="E26" s="1">
         <v>4000</v>
@@ -2038,16 +1906,16 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="B27" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E27" s="1">
         <v>23100</v>
@@ -2055,16 +1923,16 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E28" s="1">
         <v>27000</v>
@@ -2072,16 +1940,16 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="B29" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="E29" s="1">
         <v>17650</v>
@@ -2089,16 +1957,16 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="D30" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="E30" s="1">
         <v>90</v>
@@ -2106,16 +1974,16 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C31" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D31" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E31" s="1">
         <v>450</v>
@@ -2123,16 +1991,16 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B32" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="D32" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="E32" s="1">
         <v>320</v>
@@ -2140,16 +2008,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B33" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D33" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E33" s="1">
         <v>1500</v>
@@ -2157,16 +2025,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="B34" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C34" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D34" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E34" s="1">
         <v>360</v>
@@ -2187,7 +2055,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C931F77-413A-4844-949B-216B607639AF}">
   <sheetPr>
     <tabColor theme="7" tint="0.79998168889431442"/>
@@ -2207,363 +2075,363 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D1" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="6">
+        <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="6">
-        <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
-        <v>0</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>226</v>
+        <v>213</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D3" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E3" s="6">
         <v>0</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G3" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>0</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>208</v>
+        <v>195</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>226</v>
+        <v>213</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="D4" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E4" s="6">
         <v>10000</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G4" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>10000</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>200</v>
+        <v>187</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>205</v>
+        <v>192</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>201</v>
+        <v>188</v>
       </c>
       <c r="E5" s="6">
         <v>16000</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G5" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>16000</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>202</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>225</v>
+        <v>212</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D6" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E6" s="6">
         <v>1940</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G6" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>1940</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>208</v>
+        <v>195</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>225</v>
+        <v>212</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E7" s="6">
         <v>18000</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G7" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>18000</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>214</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>200</v>
+        <v>187</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>201</v>
+        <v>188</v>
       </c>
       <c r="E8" s="6">
         <v>24000</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G8" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>24000</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>203</v>
+        <v>190</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>227</v>
+        <v>214</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D9" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E9" s="6">
         <v>5710</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G9" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>5710</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>208</v>
+        <v>195</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>227</v>
+        <v>214</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="D10" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E10" s="6">
         <v>20000</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G10" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>20000</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>200</v>
+        <v>187</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>201</v>
+        <v>188</v>
       </c>
       <c r="E11" s="6">
         <v>37000</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G11" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>37000</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>228</v>
+        <v>215</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D12" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E12" s="6">
         <v>10770</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G12" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>10770</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>213</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>208</v>
+        <v>195</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>228</v>
+        <v>215</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="D13" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E13" s="6">
         <v>25000</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G13" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>25000</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>210</v>
+        <v>197</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="D14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E14" s="6">
         <v>3000</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G14" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
@@ -2572,19 +2440,19 @@
     </row>
     <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="D15" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E15" s="6">
         <v>2460</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G15" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
@@ -2593,504 +2461,504 @@
     </row>
     <row r="16" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="D16" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E16" s="6">
         <v>1051.2</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G16" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>1051.2</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="C17" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="D17" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E17" s="6">
         <v>748.15</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G17" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>748.15</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="D18" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E18" s="6">
         <v>6096.65</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G18" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>6096.65</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="C19" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="D19" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E19" s="6">
         <v>7502.9</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G19" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>7502.9</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D20" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="E20" s="6">
         <f>16750</f>
         <v>16750</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G20" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>16750</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="C21" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D21" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="E21" s="6">
         <f>887</f>
         <v>887</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G21" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>887</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="C22" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D22" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G22" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>0</v>
       </c>
       <c r="H22" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="C23" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D23" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G23" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>0</v>
       </c>
       <c r="H23" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="C24" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="D24" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="E24" s="6">
         <f>1140*12</f>
         <v>13680</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G24" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>13680</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C25" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="D25" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="E25" s="6">
         <f>2836.8*12</f>
         <v>34041.600000000006</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G25" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>34041.600000000006</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="C26" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="D26" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="E26" s="6">
         <f>1518*12</f>
         <v>18216</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G26" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>18216</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="C27" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="D27" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="E27" s="6">
         <v>516</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G27" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>516</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="C28" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="D28" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="E28" s="6">
         <v>456</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G28" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>456</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>151</v>
+        <v>138</v>
       </c>
       <c r="C29" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="D29" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E29" s="6">
         <v>660</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G29" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>660</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="C30" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D30" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E30" s="6">
         <v>2400</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G30" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>2880</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
       <c r="C31" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="D31" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E31" s="6">
         <v>2400</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G31" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>2880</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="C32" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="D32" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E32" s="6">
         <v>2450</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G32" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>2940</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="C33" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="D33" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E33" s="6">
         <v>2200</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G33" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>2640</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D34" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E34" s="6">
         <v>160</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G34" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
@@ -3099,75 +2967,75 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="C35" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="D35" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="E35" s="6">
         <f>2400*12</f>
         <v>28800</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G35" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>28800</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="C36" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="D36" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="E36" s="6">
         <f>1320*12</f>
         <v>15840</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G36" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>15840</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="D37" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E37" s="6">
         <v>3198.13</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G37" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
@@ -3176,19 +3044,19 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="D38" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E38" s="6">
         <v>3322.8</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G38" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
@@ -3197,19 +3065,19 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="D39" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E39" s="6">
         <v>3138.27</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G39" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
@@ -3218,130 +3086,130 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="C40" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D40" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E40" s="6">
         <v>240</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G40" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>288</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="C41" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="D41" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E41" s="6">
         <v>240</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G41" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>288</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="C42" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="D42" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E42" s="6">
         <v>240</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G42" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>288</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="C43" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="D43" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E43" s="6">
         <v>240</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G43" s="6">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>288</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>221</v>
+        <v>208</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="D44" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E44" s="7">
         <v>10000</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G44" s="7">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
@@ -3352,22 +3220,22 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>223</v>
+        <v>210</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E45" s="7">
         <v>12500</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G45" s="7">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
@@ -3378,22 +3246,22 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>222</v>
+        <v>209</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E46" s="7">
         <v>15000</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G46" s="7">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
@@ -3404,29 +3272,29 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="D47" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E47" s="7">
         <v>16800</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G47" s="7">
         <f>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</f>
         <v>16800</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="I47" s="2"/>
     </row>
@@ -3450,7 +3318,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC275D61-F58E-4476-8C07-B1CAEC1E0C10}">
   <sheetPr>
     <tabColor theme="2" tint="-9.9978637043366805E-2"/>
@@ -3476,75 +3344,75 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="N1" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="O1" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="P1" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="B1" t="s">
-        <v>119</v>
-      </c>
-      <c r="C1" t="s">
-        <v>120</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="J1" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>182</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="N1" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="O1" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="P1" s="10" t="s">
-        <v>187</v>
-      </c>
       <c r="Q1" s="10" t="s">
-        <v>217</v>
+        <v>204</v>
       </c>
       <c r="R1" s="10" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="S1" t="s">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="T1" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="C2" t="s">
-        <v>224</v>
+        <v>211</v>
       </c>
       <c r="D2" s="10">
         <v>217</v>
@@ -3581,13 +3449,13 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="C3" t="s">
-        <v>229</v>
+        <v>216</v>
       </c>
       <c r="D3" s="10">
         <v>82</v>
@@ -3622,13 +3490,13 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="C4" t="s">
-        <v>231</v>
+        <v>218</v>
       </c>
       <c r="D4" s="10">
         <v>102</v>
@@ -3668,13 +3536,13 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>231</v>
+        <v>218</v>
       </c>
       <c r="D5" s="10">
         <v>7</v>
@@ -3710,13 +3578,13 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="C6" t="s">
-        <v>230</v>
+        <v>217</v>
       </c>
       <c r="D6" s="10">
         <v>86</v>
@@ -3756,13 +3624,13 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C7" t="s">
-        <v>230</v>
+        <v>217</v>
       </c>
       <c r="D7" s="10">
         <v>7</v>
@@ -3803,129 +3671,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBE8C933-4065-4028-BD62-44296BEFC537}">
-  <sheetPr>
-    <tabColor theme="2" tint="-9.9978637043366805E-2"/>
-  </sheetPr>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="90.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.1796875" style="1" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="C1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1">
-        <v>-500</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1">
-        <f>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</f>
-        <v>-600</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1">
-        <v>-1500</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="1">
-        <f>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</f>
-        <v>-1800</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="1">
-        <v>-5000</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="1">
-        <f>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</f>
-        <v>-5000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" s="1">
-        <f>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="1">
-        <f>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="1">
-        <f>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="1">
-        <f>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" s="1">
-        <f>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>